<commit_message>
Complete homework 1 analysis
</commit_message>
<xml_diff>
--- a/pre-week-2/homework1.xlsx
+++ b/pre-week-2/homework1.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ceyhunugur/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ceyhunugur/Documents/DataAnalytics/pre-week-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F88FEE2B-44F4-8446-8FAE-435AD7B00298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F54627EA-B9D6-E243-A5A0-19910991095A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4320" yWindow="620" windowWidth="24480" windowHeight="16320" xr2:uid="{6968F9E8-C5C4-C94C-940F-D7465E18900B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Store_Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Store_Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -27,7 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -35,11 +35,110 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+  <si>
+    <t>Store</t>
+  </si>
+  <si>
+    <t>Monthly Sales</t>
+  </si>
+  <si>
+    <t>Store A</t>
+  </si>
+  <si>
+    <t>Store B</t>
+  </si>
+  <si>
+    <t>Store C</t>
+  </si>
+  <si>
+    <t>Store D</t>
+  </si>
+  <si>
+    <t>Store E</t>
+  </si>
+  <si>
+    <t>Store F</t>
+  </si>
+  <si>
+    <t>Store G</t>
+  </si>
+  <si>
+    <t>Store H</t>
+  </si>
+  <si>
+    <t>Store I</t>
+  </si>
+  <si>
+    <t>Store J</t>
+  </si>
+  <si>
+    <t>Store K</t>
+  </si>
+  <si>
+    <t>Store L</t>
+  </si>
+  <si>
+    <t>Statistic</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Mean</t>
+  </si>
+  <si>
+    <t>Median</t>
+  </si>
+  <si>
+    <t>Mode</t>
+  </si>
+  <si>
+    <t>Range</t>
+  </si>
+  <si>
+    <t>Std Dev</t>
+  </si>
+  <si>
+    <t>Std Dev No H</t>
+  </si>
+  <si>
+    <t>The average sales are similar for most stores.</t>
+  </si>
+  <si>
+    <t>Most values are between 43 and 52.</t>
+  </si>
+  <si>
+    <t>Store H has a much higher value than others.</t>
+  </si>
+  <si>
+    <t>It increases the average sales.</t>
+  </si>
+  <si>
+    <t>It also increases the standard deviation.</t>
+  </si>
+  <si>
+    <t>Without Store H, the data becomes more consistent.</t>
+  </si>
+  <si>
+    <t>Store H is an outlier in this dataset.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="20"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -66,8 +165,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,9 +502,210 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6125C92E-F5D5-3248-AA42-ACC5002BE06F}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>51</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2">
+        <f>AVERAGE(B2:B13)</f>
+        <v>49.416666666666664</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3">
+        <f>MEDIAN(B2:B13)</f>
+        <v>47.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>49</v>
+      </c>
+      <c r="D4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4">
+        <f>_xlfn.MODE.SNGL(B2:B13)</f>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>46</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5">
+        <f>MAX(B2:B13)-MIN(B2:B13)</f>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>52</v>
+      </c>
+      <c r="D6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6">
+        <f>_xlfn.STDEV.S(B2:B13)</f>
+        <v>7.6331613054586773</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>47</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7">
+        <f>_xlfn.STDEV.S(B2:B8,B10:B13)</f>
+        <v>2.9076701075853588</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F36DA5B-B178-D24F-89AC-C859BD26B921}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="71.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="27" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="27" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="27" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="27" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="27" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="27" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="27" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>